<commit_message>
Wire out of sample ex-post analysis to main workflow
</commit_message>
<xml_diff>
--- a/inputScenarios.xlsx
+++ b/inputScenarios.xlsx
@@ -1,45 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\01_Modelle\Simon\HeatPumpInvestment\02_IBK_case_study\base_case_v3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\OptimalHeatPumpInvestment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C85FFDC-79E5-4C36-9137-89F0FA73472C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E206E7-53FE-4935-BF29-FB8990A928DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37790" yWindow="3980" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>ScenarioIndex</t>
   </si>
@@ -47,27 +28,36 @@
     <t>InvestmentCost</t>
   </si>
   <si>
+    <t>BaseInvestmentCost</t>
+  </si>
+  <si>
+    <t>HNSCost</t>
+  </si>
+  <si>
+    <t>EHSCost</t>
+  </si>
+  <si>
+    <t>StartUpCost</t>
+  </si>
+  <si>
     <t>MinPartLoad</t>
   </si>
   <si>
-    <t>HNSCost</t>
-  </si>
-  <si>
-    <t>EHSCost</t>
-  </si>
-  <si>
     <t>StorageCapacity</t>
   </si>
   <si>
     <t>StorageSelfDischarge</t>
   </si>
   <si>
-    <t>StartUpCost</t>
+    <t>StorageChargeEfficiency</t>
   </si>
   <si>
     <t>VariableElCost</t>
   </si>
   <si>
+    <t>ElPriceScalor</t>
+  </si>
+  <si>
     <t>StartUpConstraint</t>
   </si>
   <si>
@@ -77,18 +67,24 @@
     <t>MIPGap</t>
   </si>
   <si>
+    <t>StartDay</t>
+  </si>
+  <si>
+    <t>DurationDays</t>
+  </si>
+  <si>
+    <t>InvBoundRange</t>
+  </si>
+  <si>
     <t>Units / Info</t>
   </si>
   <si>
-    <t>StartDay</t>
-  </si>
-  <si>
-    <t>DurationDays</t>
-  </si>
-  <si>
     <t>in €/kW/year</t>
   </si>
   <si>
+    <t>in  €/unit/year</t>
+  </si>
+  <si>
     <t>€/kW</t>
   </si>
   <si>
@@ -104,49 +100,31 @@
     <t>in %/h</t>
   </si>
   <si>
+    <t>in %</t>
+  </si>
+  <si>
     <t>True / False</t>
   </si>
   <si>
+    <t>rel.</t>
+  </si>
+  <si>
+    <t>0-364</t>
+  </si>
+  <si>
     <t>1-365</t>
   </si>
   <si>
-    <t>0-364</t>
+    <t>p.u.</t>
+  </si>
+  <si>
+    <t>base_case</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
   <si>
     <t xml:space="preserve">True  </t>
-  </si>
-  <si>
-    <t>InvBoundRange</t>
-  </si>
-  <si>
-    <t>p.u.</t>
-  </si>
-  <si>
-    <t>BaseInvestmentCost</t>
-  </si>
-  <si>
-    <t>in  €/unit/year</t>
-  </si>
-  <si>
-    <t>ElPriceScalor</t>
-  </si>
-  <si>
-    <t>rel.</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>in %</t>
-  </si>
-  <si>
-    <t>StorageChargeEfficiency</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>base_case</t>
   </si>
 </sst>
 </file>
@@ -520,7 +498,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -529,104 +507,104 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="R2" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B3" s="2">
         <v>128</v>
@@ -656,16 +634,16 @@
         <v>0.8</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L3" s="2">
         <v>0.8</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O3" s="2">
         <v>0.01</v>
@@ -2304,6 +2282,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update the parameter and input secnario sheet for new feature
new: numbers of segemnts, number of cores for solving
</commit_message>
<xml_diff>
--- a/inputScenarios.xlsx
+++ b/inputScenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simon Malacek\Code\OptimalHeatPumpInvestment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E206E7-53FE-4935-BF29-FB8990A928DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109D26EE-23B1-437C-98B3-1D7D72763D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37790" yWindow="3980" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38130" yWindow="3640" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
   <si>
     <t>ScenarioIndex</t>
   </si>
@@ -76,6 +76,9 @@
     <t>InvBoundRange</t>
   </si>
   <si>
+    <t>n_fit_segments</t>
+  </si>
+  <si>
     <t>Units / Info</t>
   </si>
   <si>
@@ -116,6 +119,9 @@
   </si>
   <si>
     <t>p.u.</t>
+  </si>
+  <si>
+    <t>count (PWL/PWLR secant fit)</t>
   </si>
   <si>
     <t>base_case</t>
@@ -467,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R89"/>
+  <dimension ref="A1:S89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
@@ -490,7 +496,7 @@
     <col min="18" max="18" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -545,66 +551,72 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="P2" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2">
         <v>128</v>
@@ -634,16 +646,16 @@
         <v>0.8</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L3" s="2">
         <v>0.8</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O3" s="2">
         <v>0.01</v>
@@ -657,8 +669,11 @@
       <c r="R3" s="2">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S3" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -677,8 +692,9 @@
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S4" s="2"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -697,8 +713,9 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S5" s="2"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -717,8 +734,9 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S6" s="2"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -737,8 +755,9 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S7" s="2"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -757,8 +776,9 @@
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S8" s="2"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -777,8 +797,9 @@
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S9" s="2"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -797,8 +818,9 @@
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S10" s="2"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -817,8 +839,9 @@
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S11" s="2"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -837,8 +860,9 @@
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S12" s="2"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -857,8 +881,9 @@
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S13" s="2"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -877,8 +902,9 @@
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S14" s="2"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -897,8 +923,9 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S15" s="2"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -917,8 +944,12 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="S16" s="2"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="S17" s="2"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -938,7 +969,7 @@
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -958,7 +989,7 @@
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -978,7 +1009,7 @@
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -998,7 +1029,7 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1018,7 +1049,7 @@
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1038,7 +1069,7 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1058,7 +1089,7 @@
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1078,7 +1109,7 @@
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1098,7 +1129,7 @@
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1118,7 +1149,7 @@
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1138,7 +1169,7 @@
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1158,7 +1189,7 @@
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1178,7 +1209,7 @@
       <c r="Q31" s="2"/>
       <c r="R31" s="2"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>

</xml_diff>